<commit_message>
Update LMO HULU GWP recaps from corrected SimaPro export
</commit_message>
<xml_diff>
--- a/Rekap_PROC_LMO.xlsx
+++ b/Rekap_PROC_LMO.xlsx
@@ -1265,7 +1265,9 @@
           <t>Ammonium nitrate {RoW}| market for ammonium nitrate | Cut-off, S</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n"/>
+      <c r="D10" s="2" t="n">
+        <v>1.3259296</v>
+      </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
@@ -1299,7 +1301,9 @@
     <row r="11" ht="21" customHeight="1">
       <c r="B11" s="39" t="n"/>
       <c r="C11" s="40" t="n"/>
-      <c r="D11" s="3" t="n"/>
+      <c r="D11" s="3" t="n">
+        <v>0.07160300752919138</v>
+      </c>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
@@ -1493,9 +1497,7 @@
           <t>Palm oil, crude {MY}| palm oil mill operation | Cut-off, S</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
-        <v>6.1744842</v>
-      </c>
+      <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n">
@@ -1535,9 +1537,7 @@
     <row r="19" ht="21" customHeight="1">
       <c r="B19" s="39" t="n"/>
       <c r="C19" s="40" t="n"/>
-      <c r="D19" s="3" t="n">
-        <v>0.2551598752517306</v>
-      </c>
+      <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n">
@@ -1690,7 +1690,7 @@
       <c r="B23" s="40" t="n"/>
       <c r="C23" s="40" t="n"/>
       <c r="D23" s="3" t="n">
-        <v>0.5969395117679234</v>
+        <v>0.7800625474138602</v>
       </c>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n">

</xml_diff>